<commit_message>
Remover Grupo Digital2020 dos formatos offline (dados e HTML)
O Grupo Digital2020 é uma taxonomia exclusiva dos meios digitais — não
existe nem faz sentido para publishers offline. Limpa o campo nas 27
linhas de OOH na base (data/base-formatos.xlsx) e deixa de desenhar a
coluna/etiqueta "Grupo Digital2020" em qualquer sítio do HTML para
publishers offline (Construir Pedido, Biblioteca de Formatos e resumo
da seleção) — decidido por publisher a partir do Meio, já que um
publisher pertence sempre por inteiro a um único meio.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -19446,11 +19446,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F356" t="inlineStr">
         <is>
           <t>High Impact</t>
@@ -19461,20 +19456,16 @@
           <t>Desenho técnico à escala 1/10 + 3 mm de bleed (ou na escala fornecida, no caso de veículos) — formato genérico, sem dimensão fixa.</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr"/>
-      <c r="I356" t="inlineStr"/>
       <c r="J356" t="inlineStr">
         <is>
           <t>PDF (qualidade de impressão), JPEG (visualização) e ficheiro editável (para ajustes menores)</t>
         </is>
       </c>
-      <c r="K356" t="inlineStr"/>
       <c r="L356" t="inlineStr">
         <is>
           <t>Fontes convertidas em curvas; imagens finalizadas a 300 dpi; ficheiro gravado em versão anterior à utilizada para o criar; sempre em CMYK (Pantone e RGB não aceites); sem elementos de informação relevante junto às margens de corte. Envio via WeTransfer/Hightail/Dropbox ou FTP do cliente (com utilizador e password); CD/DVD sempre com prova de cor.</t>
         </is>
       </c>
-      <c r="M356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -19497,11 +19488,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F357" t="inlineStr">
         <is>
           <t>Outdoor 8x3</t>
@@ -19512,20 +19498,16 @@
           <t>Arte final: 784x300mm (escala reduzida). Medida real: 8000x3000mm. Área visível: 7950x2950mm.</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr"/>
-      <c r="I357" t="inlineStr"/>
       <c r="J357" t="inlineStr">
         <is>
           <t>Papel cartaz 120g blueback ou AFC 120g; impressão em tintas U.V.; PDF (qualidade de impressão), JPEG (visualização) e ficheiro editável.</t>
         </is>
       </c>
-      <c r="K357" t="inlineStr"/>
       <c r="L357" t="inlineStr">
         <is>
           <t>Fontes em curvas; imagens a 300 dpi; ficheiro em versão anterior do programa; sempre CMYK (sem Pantone/RGB); sem informação relevante junto às margens de corte. Prazo de entrega: até 5 dias úteis antes do início da campanha. Cartazes entregues alceados (ordenados) e dobrados — cartaz de 14 folhas, ordem da última para a primeira folha, com a imagem voltada para cima; miras de sobreposição obrigatórias, com margens de sobreposição de 4cm do lado direito e 12,5cm no fundo das folhas inferiores (o papel tem distensão variável). Quantidades: Abril a Setembro, +15% do nº de faces; Outubro a Março, +25%. Cartazes entregues e identificados à unidade, e alceados. Nota: imagens com fundos escuros ou que necessitem de muita tinta reduzem a qualidade da afixação. Envio via WeTransfer/Hightail/Dropbox ou FTP do cliente; CD/DVD sempre com prova de cor.</t>
         </is>
       </c>
-      <c r="M357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -19548,11 +19530,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
-        <is>
-          <t>Multibanco</t>
-        </is>
-      </c>
       <c r="F358" t="inlineStr">
         <is>
           <t>Multibanco - Imagem</t>
@@ -19563,7 +19540,6 @@
           <t>3 tamanhos disponíveis: 640x417px, 800x522px ou 1024x667px. 3 momentos distintos: 1º momento 10s, 2º momento 3s, 3º momento 10s (pode usar 1, 2 ou 3 imagens diferentes, ou combinar com vídeo nos vários momentos).</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
       <c r="I358" t="inlineStr">
         <is>
           <t>Máx. 1 MB</t>
@@ -19574,13 +19550,11 @@
           <t>JPG ou PNG, resolução igual ou superior a 72 dpi</t>
         </is>
       </c>
-      <c r="K358" t="inlineStr"/>
       <c r="L358" t="inlineStr">
         <is>
           <t>Não é possível apresentar conteúdos que mostrem, de forma explícita e não contextualizada, partes do corpo habitualmente resguardadas; mencionem instituições financeiras monetárias e de pagamento, partidos/associações políticas ou sindicais, organizações religiosas; usem símbolos/linguagem que se possam confundir com o funcionamento do caixa automático; ou que, no primeiro momento publicitário, mostrem qualquer preço sem identificação clara de que é um preço do anunciante, produto ou serviço. Para todos os outros princípios aplica-se o código da publicidade.</t>
         </is>
       </c>
-      <c r="M358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -19603,11 +19577,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr">
-        <is>
-          <t>Multibanco</t>
-        </is>
-      </c>
       <c r="F359" t="inlineStr">
         <is>
           <t>Multibanco - Vídeo</t>
@@ -19618,7 +19587,6 @@
           <t>2 tamanhos disponíveis: 640x392px ou 800x496px. 3 momentos distintos: 1º momento 5s, 2º momento 2s, 3º momento 5s (pode usar 1, 2 ou 3 vídeos diferentes, ou combinar com imagens nos vários momentos; sugestão: terminar com a imagem estática do último frame).</t>
         </is>
       </c>
-      <c r="H359" t="inlineStr"/>
       <c r="I359" t="inlineStr">
         <is>
           <t>Máx. 1 MB</t>
@@ -19629,13 +19597,11 @@
           <t>MPEG-1 ou MP4</t>
         </is>
       </c>
-      <c r="K359" t="inlineStr"/>
       <c r="L359" t="inlineStr">
         <is>
           <t>Sem canal áudio. Frame rate: 24 frames/s. Profundidade de cor: 24 bits/pixel. Mesmos princípios de conteúdo do formato "Multibanco - Imagem".</t>
         </is>
       </c>
-      <c r="M359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -19658,11 +19624,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr">
-        <is>
-          <t>Decoração</t>
-        </is>
-      </c>
       <c r="F360" t="inlineStr">
         <is>
           <t>Decorações Integrais e Grande Formato</t>
@@ -19673,20 +19634,16 @@
           <t>Desenho técnico à escala 1/10 + 3 mm de bleed (ou na escala fornecida, no caso de veículos).</t>
         </is>
       </c>
-      <c r="H360" t="inlineStr"/>
-      <c r="I360" t="inlineStr"/>
       <c r="J360" t="inlineStr">
         <is>
           <t>PDF (qualidade de impressão), JPEG (visualização) e ficheiro editável (para ajustes menores)</t>
         </is>
       </c>
-      <c r="K360" t="inlineStr"/>
       <c r="L360" t="inlineStr">
         <is>
           <t>Fontes convertidas em curvas; imagens finalizadas a 300 dpi; ficheiro gravado em versão anterior do programa; sempre CMYK (sem Pantone/RGB); sem informação relevante junto às margens de corte. Envio via WeTransfer/Hightail/Dropbox ou FTP do cliente; CD/DVD sempre com prova de cor.</t>
         </is>
       </c>
-      <c r="M360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -19709,11 +19666,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr">
-        <is>
-          <t>LED Indoor</t>
-        </is>
-      </c>
       <c r="F361" t="inlineStr">
         <is>
           <t>Grande Formato Digital Indoor 16x9</t>
@@ -19739,13 +19691,11 @@
           <t>MP4, codec H264</t>
         </is>
       </c>
-      <c r="K361" t="inlineStr"/>
       <c r="L361" t="inlineStr">
         <is>
           <t>Duração: 10 segundos (obrigatório). Bitrate máx. 6 Mbps. Framerate 24 frames/s. No suporte de 3 ecrãs existe uma separação real de 2,5cm entre ecrãs, que divide/corta a imagem — deve ser tido em conta para não deformar frases ou elementos relevantes (zonas de quebra).</t>
         </is>
       </c>
-      <c r="M361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -19768,11 +19718,6 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr">
-        <is>
-          <t>Mupi</t>
-        </is>
-      </c>
       <c r="F362" t="inlineStr">
         <is>
           <t>Mupi Digital</t>
@@ -19798,13 +19743,11 @@
           <t>MP4, codec H264</t>
         </is>
       </c>
-      <c r="K362" t="inlineStr"/>
       <c r="L362" t="inlineStr">
         <is>
           <t>Duração: 10 segundos (obrigatório). Bitrate máx. 6 Mbps. Framerate 24 frames/s.</t>
         </is>
       </c>
-      <c r="M362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -19827,35 +19770,26 @@
           <t>MOP</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr">
+      <c r="F363" t="inlineStr">
         <is>
           <t>Mupi</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr">
-        <is>
-          <t>Mupi</t>
-        </is>
-      </c>
       <c r="G363" t="inlineStr">
         <is>
           <t>Arte final: 234x348mm + 1mm de bleed. Medida real: 1185x1750mm. Área visível: 1131x1667mm.</t>
         </is>
       </c>
-      <c r="H363" t="inlineStr"/>
-      <c r="I363" t="inlineStr"/>
       <c r="J363" t="inlineStr">
         <is>
           <t>PDF (qualidade de impressão), JPEG (visualização) e ficheiro editável</t>
         </is>
       </c>
-      <c r="K363" t="inlineStr"/>
       <c r="L363" t="inlineStr">
         <is>
           <t>Fontes em curvas; imagens a 300 dpi; ficheiro em versão anterior do programa; sempre CMYK (sem Pantone/RGB); sem informação relevante junto às margens de corte. Envio via WeTransfer/Hightail/Dropbox ou FTP do cliente; CD/DVD sempre com prova de cor.</t>
         </is>
       </c>
-      <c r="M363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -19878,11 +19812,6 @@
           <t>DreamMedia</t>
         </is>
       </c>
-      <c r="E364" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F364" t="inlineStr">
         <is>
           <t>Outdoor 8x3</t>
@@ -19893,20 +19822,16 @@
           <t>8000x3000mm (área de mancha publicitária = área visível).</t>
         </is>
       </c>
-      <c r="H364" t="inlineStr"/>
-      <c r="I364" t="inlineStr"/>
       <c r="J364" t="inlineStr">
         <is>
           <t>Ficheiro fechado: JPG, TIFF ou PDF, a 10% do tamanho real, a 300 dpi. Formato editável: textos convertidos em curvas (outlines) ou fontes fornecidas.</t>
         </is>
       </c>
-      <c r="K364" t="inlineStr"/>
       <c r="L364" t="inlineStr">
         <is>
           <t>Bleed: 10cm a toda a volta (não deve conter informação importante). Ficheiros fornecidos em CMYK prontos para impressão — ficheiros em RGB são convertidos para CMYK, podendo as cores sofrer alterações.</t>
         </is>
       </c>
-      <c r="M364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -19929,11 +19854,6 @@
           <t>BIG Outdoors</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F365" t="inlineStr">
         <is>
           <t>Monoposte 10x5</t>
@@ -19944,20 +19864,16 @@
           <t>Área de mancha publicitária: 10000x5000mm.</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr"/>
-      <c r="I365" t="inlineStr"/>
       <c r="J365" t="inlineStr">
         <is>
           <t>Ficheiro fechado: JPG, TIFF ou PDF, a 10% do tamanho real, a 300 dpi. Formato editável: textos convertidos em curvas (outlines) ou fontes fornecidas.</t>
         </is>
       </c>
-      <c r="K365" t="inlineStr"/>
       <c r="L365" t="inlineStr">
         <is>
           <t>Bleed: 10cm a toda a volta (não deve conter informação importante). Ficheiros fornecidos em CMYK prontos para impressão — ficheiros em RGB são convertidos para CMYK, podendo as cores sofrer alterações. Importante: a arte final não deve conter letras de tamanho inferior a 30cm (110 pontos); dar maior destaque ao produto, logótipo, telefone e site para melhores resultados de comunicação.</t>
         </is>
       </c>
-      <c r="M365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -19980,11 +19896,6 @@
           <t>BIG Outdoors</t>
         </is>
       </c>
-      <c r="E366" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F366" t="inlineStr">
         <is>
           <t>Monoposte 11x5</t>
@@ -19995,20 +19906,16 @@
           <t>Área de mancha publicitária: 11000x5000mm.</t>
         </is>
       </c>
-      <c r="H366" t="inlineStr"/>
-      <c r="I366" t="inlineStr"/>
       <c r="J366" t="inlineStr">
         <is>
           <t>Ficheiro fechado: JPG, TIFF ou PDF, a 10% do tamanho real, a 300 dpi. Formato editável: textos convertidos em curvas (outlines) ou fontes fornecidas.</t>
         </is>
       </c>
-      <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr">
         <is>
           <t>Bleed: 10cm a toda a volta (não deve conter informação importante). Ficheiros fornecidos em CMYK prontos para impressão — ficheiros em RGB são convertidos para CMYK, podendo as cores sofrer alterações. Importante: a arte final não deve conter letras de tamanho inferior a 30cm (110 pontos); dar maior destaque ao produto, logótipo, telefone e site para melhores resultados de comunicação.</t>
         </is>
       </c>
-      <c r="M366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -20031,11 +19938,6 @@
           <t>BIG Outdoors</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F367" t="inlineStr">
         <is>
           <t>Monoposte 12x5</t>
@@ -20046,20 +19948,16 @@
           <t>Área de mancha publicitária: 12000x5000mm.</t>
         </is>
       </c>
-      <c r="H367" t="inlineStr"/>
-      <c r="I367" t="inlineStr"/>
       <c r="J367" t="inlineStr">
         <is>
           <t>Ficheiro fechado: JPG, TIFF ou PDF, a 10% do tamanho real, a 300 dpi. Formato editável: textos convertidos em curvas (outlines) ou fontes fornecidas.</t>
         </is>
       </c>
-      <c r="K367" t="inlineStr"/>
       <c r="L367" t="inlineStr">
         <is>
           <t>Bleed: 10cm a toda a volta (não deve conter informação importante). Ficheiros fornecidos em CMYK prontos para impressão — ficheiros em RGB são convertidos para CMYK, podendo as cores sofrer alterações. Importante: a arte final não deve conter letras de tamanho inferior a 30cm (110 pontos); dar maior destaque ao produto, logótipo, telefone e site para melhores resultados de comunicação.</t>
         </is>
       </c>
-      <c r="M367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -20082,11 +19980,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr">
-        <is>
-          <t>Mupi</t>
-        </is>
-      </c>
       <c r="F368" t="inlineStr">
         <is>
           <t>Mupi Papel</t>
@@ -20097,20 +19990,16 @@
           <t>Área total: 1185x1750mm. Área visível: 1160x1710mm.</t>
         </is>
       </c>
-      <c r="H368" t="inlineStr"/>
-      <c r="I368" t="inlineStr"/>
       <c r="J368" t="inlineStr">
         <is>
           <t>Papel, gramagem 130g, verso do cartaz com fundo branco. Ficheiro: Illustrator, Photoshop, PDF, EPS ou TIFF.</t>
         </is>
       </c>
-      <c r="K368" t="inlineStr"/>
       <c r="L368" t="inlineStr">
         <is>
           <t>Prazo: 7 dias úteis após aprovação da Arte Final. Se enviar PDF, atenção a cores/perfis embebidos/resolução de imagens; enviar fontes; texto convertido em curvas, aberto e editável. Impressão offset: CMYK, mín. 300 dpi, máx. 400 dpi. Impressão digital: CMYK, mín. 150 dpi, máx. 200 dpi. Ficheiro na medida indicada + 3cm de bleed (3mm se a AF for elaborada à escala de 10%); respeitar área de segurança virtual para evitar corte de elementos na afixação; sempre que possível, enviar com prova de cor. Após receção, a JCDecaux envia um JPG para validação final antes de imprimir; após aprovação, declina responsabilidade por desformatações/falhas na imagem. Critérios de qualidade: opacidade ≥88%, brancura 91-93 ISO, absorção de água (cobb60) 15-30g/m², absorção de água (cobb300) &lt;70g/m², distensão máx. ±2%/m, resistência à rutura por tração (húmido) &gt;0,6kN/m — materiais fora destes requisitos podem não ser afixados. Especificações ambientais: papel com certificação PEFC/FSC (ou equivalente); tintas conformes REACH/GreenGuard, isentas de metais pesados; papel reciclado, sem cloro (ECF/TCF).</t>
         </is>
       </c>
-      <c r="M368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -20133,11 +20022,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F369" t="inlineStr">
         <is>
           <t>Impressão Senior</t>
@@ -20148,20 +20032,16 @@
           <t>Área visível: 3020x2230mm. Área total: 3200x2350mm.</t>
         </is>
       </c>
-      <c r="H369" t="inlineStr"/>
-      <c r="I369" t="inlineStr"/>
       <c r="J369" t="inlineStr">
         <is>
           <t>Papel, gramagem 150g, verso do cartaz com fundo branco. Ficheiro: Illustrator, Photoshop, PDF, EPS ou TIFF.</t>
         </is>
       </c>
-      <c r="K369" t="inlineStr"/>
       <c r="L369" t="inlineStr">
         <is>
           <t>Impressão em 1, 2 ou 4 folhas, entregues alceadas por ordem de colagem (a começar na folha 1, com o verso para baixo). Impressão em 2 folhas: folha 1 3200x1200mm (aparada 3130x1150mm) + folha 2 idêntica, margem de sobreposição 25mm/35mm. Impressão em 4 folhas: 1600x1200mm por folha (aparada 1530x1175mm), aparadas à medida sem margem entre si. Prazo: 7 dias úteis após aprovação da Arte Final. Ficheiro: Illustrator/Photoshop (incluir fontes e respetivos links) ou PDF (cores/perfis embebidos/resolução de imagens, texto em curvas); impressão offset CMYK 300-400 dpi, digital CMYK 150-200 dpi; medida indicada + 3cm de bleed (3mm à escala de 10%); respeitar área de segurança virtual; enviar com prova de cor sempre que possível. Entrega nas instalações da JCDecaux 5 dias úteis antes do início da campanha, com impressão da campanha e guia de transporte certificada; horário de entrega 07h-12h e 13h30-16h (Portão 2), Beco da Aviação nº1, Granja do Alpriate, Vialonga. Após receção, a JCDecaux envia JPG para validação; após aprovação, declina responsabilidade por falhas na imagem. Critérios de qualidade: opacidade ≥88%, brancura 91-93 ISO, absorção água (cobb60) 15-30g/m², (cobb300) &lt;70g/m², distensão máx. ±2%/m, resistência à rutura (húmido) &gt;0,6kN/m.</t>
         </is>
       </c>
-      <c r="M369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -20184,11 +20064,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr">
-        <is>
-          <t>Mupi</t>
-        </is>
-      </c>
       <c r="F370" t="inlineStr">
         <is>
           <t>Mupi Digital</t>
@@ -20204,19 +20079,16 @@
           <t>9:16</t>
         </is>
       </c>
-      <c r="I370" t="inlineStr"/>
       <c r="J370" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K370" t="inlineStr"/>
       <c r="L370" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Após envio, a JCDecaux declina responsabilidade por falhas no vídeo apresentado. Alterações ao vídeo carecem de aprovação final do cliente; a JCDecaux não se responsabiliza por atraso na entrega (sem compensação de airing).</t>
         </is>
       </c>
-      <c r="M370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -20239,11 +20111,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr">
-        <is>
-          <t>Mupi</t>
-        </is>
-      </c>
       <c r="F371" t="inlineStr">
         <is>
           <t>Mupi Digital (Shopping)</t>
@@ -20259,19 +20126,16 @@
           <t>16:9 (ficheiro) / 9:16 (exibição)</t>
         </is>
       </c>
-      <c r="I371" t="inlineStr"/>
       <c r="J371" t="inlineStr">
         <is>
           <t>Ficheiro nativo (compressão nativa), bitrate máx. 20.000.</t>
         </is>
       </c>
-      <c r="K371" t="inlineStr"/>
       <c r="L371" t="inlineStr">
         <is>
           <t>Duração do spot: 10 segundos, dentro de um loop de 60 segundos com outros anunciantes. Enviar o vídeo 2 dias antes do início da campanha, por e-mail para o contacto JCDecaux. Alterações carecem de aprovação final do cliente; a JCDecaux declina responsabilidade por falhas no vídeo após o envio, e não se responsabiliza por atraso na entrega.</t>
         </is>
       </c>
-      <c r="M371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -20294,11 +20158,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F372" t="inlineStr">
         <is>
           <t>Painel 8x3 - Papel</t>
@@ -20309,20 +20168,16 @@
           <t>Área total: 8000x3000mm. Área visível: 7500x2750mm.</t>
         </is>
       </c>
-      <c r="H372" t="inlineStr"/>
-      <c r="I372" t="inlineStr"/>
       <c r="J372" t="inlineStr">
         <is>
           <t>Papel, gramagem entre 120g e 170g, verso do cartaz com fundo azul. Ficheiro: Illustrator, Photoshop, PDF, EPS ou TIFF.</t>
         </is>
       </c>
-      <c r="K372" t="inlineStr"/>
       <c r="L372" t="inlineStr">
         <is>
           <t>Prazo: 7 dias úteis após aprovação da Arte Final. Impressão em 12, 14 ou 16 folhas, entregues alceadas (a começar na folha 1, verso para baixo), numeradas no canto superior direito. Impressão em 14 folhas: folhas superiores 1-6 (997mm cada) + folha 7 (997mm), folhas inferiores 9-13 (1135mm cada) + folha 14 (1135mm); margem de sobreposição 25mm à direita nas folhas superiores (exceto a última) e 25mm à direita + no topo nas inferiores (exceto a última, só no topo); áreas de sobreposição isentas de impressão. Impressão em 16 folhas: superiores 1-7 (997mm) + folha 8 (997mm), inferiores 9-15 (997mm) + folha 16 (997mm), mesmas regras de margem. Se PDF: cores/perfis embebidos/resolução de imagens, texto em curvas; impressão offset CMYK 300-400 dpi, digital CMYK 150-200 dpi; medida indicada + 3cm de bleed (3mm à escala de 10%); área de segurança virtual; prova de cor recomendada. Entrega nas instalações JCDecaux, Portão 1, Beco da Aviação nº1, Granja do Alpriate, Vialonga, 07h-12h/13h30-16h. Após receção, JCDecaux envia JPG para validação; após aprovação, declina responsabilidade por falhas na imagem.</t>
         </is>
       </c>
-      <c r="M372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -20345,11 +20200,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E373" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F373" t="inlineStr">
         <is>
           <t>Painel 8x3 - Vinil</t>
@@ -20360,20 +20210,16 @@
           <t>Área total: 8000x3000mm. Área visível: 8000x3000mm (sem margem).</t>
         </is>
       </c>
-      <c r="H373" t="inlineStr"/>
-      <c r="I373" t="inlineStr"/>
       <c r="J373" t="inlineStr">
         <is>
           <t>Vinil PVC branco ou transparente, superfície brilhante ou mate, polyacrylate removível e transparente; base em papel revestido a silicone 135g/m². Ficheiro: Illustrator, Photoshop, PDF, EPS ou TIFF.</t>
         </is>
       </c>
-      <c r="K373" t="inlineStr"/>
       <c r="L373" t="inlineStr">
         <is>
           <t>Uso recomendado: outdoors de curta e média duração. Método de impressão: tintas de base solvente, UV ou látex. Prazo: 7 dias úteis após aprovação da Arte Final. Impressão em 8 folhas de 1000mm cada, enroladas por ordem (folha 1 a 8), numeradas no canto superior direito; margem de sobreposição 25mm à direita em todas as folhas (áreas de sobreposição isentas de impressão). Se PDF: cores/perfis embebidos/resolução de imagens, texto em curvas; impressão offset CMYK 300-400 dpi, digital CMYK 150-200 dpi; medida indicada + 5cm de bleed (5mm à escala de 10%); área de segurança virtual; prova de cor recomendada. Entrega nas instalações JCDecaux, Portão 1, Beco da Aviação nº1, Granja do Alpriate, Vialonga, 5 dias úteis antes do início da campanha, com impressão da campanha e guia de transporte certificada, 07h-12h/13h30-16h. Após receção, JCDecaux envia JPG para validação; após aprovação, declina responsabilidade por falhas na imagem.</t>
         </is>
       </c>
-      <c r="M373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -20396,11 +20242,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E374" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F374" t="inlineStr">
         <is>
           <t>Premium LED 6m²</t>
@@ -20416,19 +20257,16 @@
           <t>2:3</t>
         </is>
       </c>
-      <c r="I374" t="inlineStr"/>
       <c r="J374" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K374" t="inlineStr"/>
       <c r="L374" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 4 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -20451,11 +20289,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E375" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F375" t="inlineStr">
         <is>
           <t>Premium LED 8m²</t>
@@ -20471,19 +20304,16 @@
           <t>9:16</t>
         </is>
       </c>
-      <c r="I375" t="inlineStr"/>
       <c r="J375" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K375" t="inlineStr"/>
       <c r="L375" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -20506,11 +20336,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E376" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F376" t="inlineStr">
         <is>
           <t>Premium LED 12m²</t>
@@ -20526,19 +20351,16 @@
           <t>1.91:1</t>
         </is>
       </c>
-      <c r="I376" t="inlineStr"/>
       <c r="J376" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -20561,11 +20383,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F377" t="inlineStr">
         <is>
           <t>Premium LED 15m²</t>
@@ -20581,19 +20398,16 @@
           <t>9:16</t>
         </is>
       </c>
-      <c r="I377" t="inlineStr"/>
       <c r="J377" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K377" t="inlineStr"/>
       <c r="L377" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -20616,11 +20430,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E378" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F378" t="inlineStr">
         <is>
           <t>Premium LED 18m²</t>
@@ -20636,19 +20445,16 @@
           <t>9:16</t>
         </is>
       </c>
-      <c r="I378" t="inlineStr"/>
       <c r="J378" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K378" t="inlineStr"/>
       <c r="L378" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -20671,11 +20477,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F379" t="inlineStr">
         <is>
           <t>Premium LED 22m²</t>
@@ -20686,20 +20487,16 @@
           <t>1248x800px.</t>
         </is>
       </c>
-      <c r="H379" t="inlineStr"/>
-      <c r="I379" t="inlineStr"/>
       <c r="J379" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K379" t="inlineStr"/>
       <c r="L379" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. Vídeo em estilo "Subtle Motion" recomendado: movimento lento e gradual dos elementos criativos (slow motion sem cortes bruscos; fundos deslocados/ampliados lentamente em vez de intermitentes; texto a desvanecer gradualmente em vez de deslizar/pulsar; luzes a brilhar em vez de piscar); marca visível em pelo menos 80% da criatividade. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -20722,11 +20519,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F380" t="inlineStr">
         <is>
           <t>Premium LED 25m²</t>
@@ -20737,20 +20529,16 @@
           <t>480x810px.</t>
         </is>
       </c>
-      <c r="H380" t="inlineStr"/>
-      <c r="I380" t="inlineStr"/>
       <c r="J380" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K380" t="inlineStr"/>
       <c r="L380" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 12,5%. A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -20773,11 +20561,6 @@
           <t>JCDecaux</t>
         </is>
       </c>
-      <c r="E381" t="inlineStr">
-        <is>
-          <t>Billboard</t>
-        </is>
-      </c>
       <c r="F381" t="inlineStr">
         <is>
           <t>Premium LED 37m²</t>
@@ -20788,20 +20571,16 @@
           <t>480x738px.</t>
         </is>
       </c>
-      <c r="H381" t="inlineStr"/>
-      <c r="I381" t="inlineStr"/>
       <c r="J381" t="inlineStr">
         <is>
           <t>Quicktime (.MOV) ou .MP4, codec H264, compressão nativa, bitrate entre 6.000 e 20.000.</t>
         </is>
       </c>
-      <c r="K381" t="inlineStr"/>
       <c r="L381" t="inlineStr">
         <is>
           <t>Framerate 25fps; duração 10 seg.; sem canal áudio. Envio do vídeo 2 dias úteis antes do início da campanha, por e-mail para o contacto JCDecaux. Share of time: 16,7%. Vídeo em estilo "Subtle Motion" recomendado (ver formato "Premium LED 22m²" para guidelines completas). A JCDecaux declina responsabilidade por falhas no vídeo após o envio; não se responsabiliza por atraso na entrega (sem compensação de airing); alterações carecem de aprovação final do cliente.</t>
         </is>
       </c>
-      <c r="M381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -20824,11 +20603,6 @@
           <t>Táxi Advertising</t>
         </is>
       </c>
-      <c r="E382" t="inlineStr">
-        <is>
-          <t>Decoração</t>
-        </is>
-      </c>
       <c r="F382" t="inlineStr">
         <is>
           <t>Decoração de Táxi</t>
@@ -20839,20 +20613,16 @@
           <t>Manter o tamanho original do template (ficheiros vetoriais reais fornecidos pelo fornecedor, com o desenho do lado esquerdo e do lado direito do táxi).</t>
         </is>
       </c>
-      <c r="H382" t="inlineStr"/>
-      <c r="I382" t="inlineStr"/>
       <c r="J382" t="inlineStr">
         <is>
           <t>Ficheiros de trabalho em Illustrator (vetoriais). Entrega: JPG ou PDF.</t>
         </is>
       </c>
-      <c r="K382" t="inlineStr"/>
       <c r="L382" t="inlineStr">
         <is>
           <t>O texto deve manter-se dentro da linha amarela de segurança (para não ser cortado). O fundo atrás do texto deve ultrapassar a linha branca em pelo menos 50mm de bleed. Impressão em CMYK, resolução 150 pixels/polegada. É obrigatório enviar também um PDF com a maqueta da decoração do táxi, para orientação da colagem do vinil.</t>
         </is>
       </c>
-      <c r="M382" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sheet extra por formato de OOH com a imagem técnica e as medidas
Acrescenta a coluna "Imagem" à base-formatos.xlsx (caminho para um PNG
com o desenho técnico/medidas do formato) — opcional, só para OOH. Cada
formato de OOH selecionado que tenha essa coluna preenchida ganha, além
da folha normal de OOH, a sua própria sheet extra no Excel exportado,
com a imagem (à escala, mantendo a proporção) e a Dimensão por baixo —
pedido explícito da Cláudia, para servir de referência de produção tal
como as fotos cotadas que fornecedores como a JCDecaux costumam enviar.

Formatos sem imagem associada não geram sheet nenhuma — a coluna fica
vazia por agora em todas as linhas, a preencher fornecedor a fornecedor
conforme formos recebendo as imagens.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M762"/>
+  <dimension ref="A1:N762"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,11 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Link</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Imagem</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Programático: renomeia fornecedor DV360 para Havas Programmatic Hub
Afeta os 18 formatos de Programático que tinham DV360 como Fornecedor
(standard banners, pre-roll, outstream, YouTube, Uber Journey Ad, ...).
O Veículo de cada um mantém-se tal como estava (DV360, YouTube, Uber) —
só o nome do fornecedor/secção que aparece na lista de seleção e nas
chaves de tradução muda. Chaves de traducoes-specs.json atualizadas em
conformidade, para as specs em EN/ES/FR continuarem a aparecer.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -11674,7 +11674,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -11778,7 +11778,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -11934,7 +11934,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -14168,7 +14168,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -14220,7 +14220,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -14277,7 +14277,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -14309,7 +14309,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>DV360</t>
+          <t>Havas Programmatic Hub</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona fornecedor Ad Click e formato Interstitial Mobile/Splash
Novo fornecedor Ad Click, com o formato Interstitial Mobile/Splash
(mobile, overlay de alto impacto que esconde o conteúdo da página,
fecha ao fim de 5s ou por botão skip; imagens 640x960 ou 800x600px,
JPG/PNG/GIF, máx. 200 KB).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N907"/>
+  <dimension ref="A1:N908"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43184,6 +43184,53 @@
         </is>
       </c>
     </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Ad Click</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Ad Click</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>Interstitial Mobile/Splash</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>Imagem: 640x960px ou 800x600px.</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>Máx. 200 KB (imagens). Duração: 5 segundos.</t>
+        </is>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>JPG, PNG ou GIF</t>
+        </is>
+      </c>
+      <c r="L908" t="inlineStr">
+        <is>
+          <t>Formato de Alto Impacto, mobile — sobrepõe-se à página através de um overlay que esconde todo o conteúdo; fecha automaticamente ao fim de 5 segundos ou através do botão skip. Não é um formato responsive. Cumprir specs SAPO (funcionalidades, peso, ações). Permitir contagem de clicks com a variável ${CLICK_URL_ENC}. Enviar em https. Incluir botão fechar (IAB). Enviar tag complementar que fecha apenas por ação do utilizador.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>